<commit_message>
Scrub residual MQTT mentions from five asset rows
Remove MQTT from current-state claims in assets 10, 18, 28, 35, 41 and add a
one-line out-of-scope future note on transport/endpoint rows so the claim is
not re-introduced.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0158eT26M2Dsi3JDmdySDo5Y
</commit_message>
<xml_diff>
--- a/en18031_asset_inventory/merged_for_import_2026-10-02.xlsx
+++ b/en18031_asset_inventory/merged_for_import_2026-10-02.xlsx
@@ -582,7 +582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A44"/>
+  <dimension ref="A1:A45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="150" customWidth="1" style="26" min="1" max="1"/>
@@ -791,35 +791,35 @@
     </row>
     <row r="33" ht="15.75" customHeight="1" s="26"/>
     <row r="34" ht="15.75" customHeight="1" s="26">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="0" t="inlineStr">
         <is>
           <t>CHANGELOG — Revision 2 (9/25/26)</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1" s="26">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="0" t="inlineStr">
         <is>
           <t>1. CORRECTION: 'MQTT' credentials/transport retracted from rows 4, 24, 33, 53 on the Asset Inventory sheet. That architecture (Event Bus over MQTT, MQTT User Biometrics, Apple Watch MQTT Transport Confluence pages) is a proposed FUTURE ToG (Tailor on Glass) tablet project, not current Valinor implementation — flagged by Dave Christensen after live review with the CSA consultant. Actual current telemetry transport mechanism is now an open GAP.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="26">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="0" t="inlineStr">
         <is>
           <t>2. NEW SOURCE: iFIT's official NIST IR 8259A response to CSA Group (Mindi Strong to Albert Bennett, 9/25/26, Project 80308127, Eway Xenon1 Tablet) — the first ENGINEERING-CONFIRMED, submitted-to-certifier source in this register. Rows updated: 5 (credential storage path/mechanism confirmed), 8 (kiosk lockdown corroboration), 9 (partial — USB debugging lockdown, but hardcoded-credential question still open), 10 (AVB/verified boot CONFIRMED for Xenon1/Eway specifically), 14 (anti-rollback CONFIRMED for Xenon1/Eway, software/timestamp-layer), 15 (auth lockout thresholds RESOLVED), 17 (OTA + APK signature verification RESOLVED for Xenon1/Eway), 20 (backup/extraction controls added), 41 (partially addressed — HTTP log redaction confirmed, CS-log PII exposure still open).</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1" s="26">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="0" t="inlineStr">
         <is>
           <t>3. IMPORTANT SCOPE NUANCE: the NIST 8259A response is specific to the Eway-built Xenon1 tablet. Several 'RESOLVED' items above apply to that variant only — Xenon-V, Xenon1.2, and Cesium are NOT automatically covered by the same confirmation and remain open per their original GAP status unless separately confirmed.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="26">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="0" t="inlineStr">
         <is>
           <t>4. Zero rows in this register carry engineering sign-off beyond what's captured above — everything else remains sourced from Confluence/Jira documentation review, not validated by iFIT engineering or accepted by CSA Group.</t>
         </is>
@@ -827,7 +827,7 @@
     </row>
     <row r="39" ht="15.75" customHeight="1" s="26"/>
     <row r="40" ht="15.75" customHeight="1" s="26">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="0" t="inlineStr">
         <is>
           <t>Pending: console/SKU priority test list (attached 9/25/26) not yet cross-referenced into this register.</t>
         </is>
@@ -835,27 +835,33 @@
     </row>
     <row r="41" ht="15.75" customHeight="1" s="26"/>
     <row r="42" ht="15.75" customHeight="1" s="26">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="0" t="inlineStr">
         <is>
           <t>CHANGELOG — Revision 3 (10/2/26)</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1" s="26">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="0" t="inlineStr">
         <is>
           <t>1. Merged Revision 2 corrections (items 1–4 above) into this live sheet. Only the corrected cells were ported: Asset Inventory rows 5, 8, 9, 10, 14, 15, 17, 20, 25, 34, 56 (cols B/K/L/M as applicable). All reviewer edits made directly in this sheet since 9/18/26 (asset 1 annotations, candidate assets rows 60–66, scoping notes rows 74–77, Interfaces rows 14–18, ArcX note) were preserved unchanged.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1" s="26">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="0" t="inlineStr">
         <is>
           <t>2. Source of truth is now this Google Sheet; a git-tracked snapshot (xlsx + per-tab CSV) is kept in the claude_scratch repo under en18031_asset_inventory/.</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="15.75" customHeight="1" s="26"/>
+    <row r="45" ht="15.75" customHeight="1" s="26">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>3. Residual MQTT mentions scrubbed from Asset Inventory rows 11, 19, 29, 36, 42 (assets 10, 18, 28, 35, 41). Current product does not use MQTT. Where a transport/endpoint cell is concerned, a one-line 'Future note' records that a proposed ToG project may add an MQTT-like service, explicitly out of current scope, so the claim is not re-introduced by mistake.</t>
+        </is>
+      </c>
+    </row>
     <row r="46" ht="15.75" customHeight="1" s="26"/>
     <row r="47" ht="15.75" customHeight="1" s="26"/>
     <row r="48" ht="15.75" customHeight="1" s="26"/>
@@ -2518,7 +2524,7 @@
       </c>
       <c r="L11" s="12" t="inlineStr">
         <is>
-          <t>HTTPS/GraphQL API; MQTT-over-TLS.</t>
+          <t>HTTPS/GraphQL API (TLS). Future note: a proposed ToG tablet project may add an MQTT-like pub/sub service; NOT in current Xenon/Cesium scope and excluded from this assessment.</t>
         </is>
       </c>
       <c r="M11" s="12" t="inlineStr">
@@ -3004,12 +3010,12 @@
       <c r="J19" s="10" t="n"/>
       <c r="K19" s="12" t="inlineStr">
         <is>
-          <t>Android framework BoringSSL; Valinor OkHttp / MQTT client libraries.</t>
+          <t>Android framework BoringSSL; Valinor OkHttp client library.</t>
         </is>
       </c>
       <c r="L19" s="12" t="inlineStr">
         <is>
-          <t>All TLS connections (GraphQL HTTPS, MQTT-over-TLS).</t>
+          <t>All TLS connections (GraphQL HTTPS). Future note: a proposed ToG tablet project may add an MQTT-like pub/sub service; NOT in current Xenon/Cesium scope and excluded from this assessment.</t>
         </is>
       </c>
       <c r="M19" s="12" t="inlineStr">
@@ -3574,7 +3580,7 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>Cloud endpoint / MQTT broker URL</t>
+          <t>Cloud endpoint URL(s)</t>
         </is>
       </c>
       <c r="C29" s="18" t="inlineStr">
@@ -3615,7 +3621,7 @@
       <c r="J29" s="18" t="n"/>
       <c r="K29" s="12" t="inlineStr">
         <is>
-          <t>Valinor BuildConfig / remote config; not user-editable in production builds.</t>
+          <t>Valinor BuildConfig / remote config; not user-editable in production builds. (Prior 'MQTT broker URL' wording retracted 10/2/26 — no broker in current product. Future note: a proposed ToG tablet project may add an MQTT-like pub/sub service; NOT in current Xenon/Cesium scope and excluded from this assessment.)</t>
         </is>
       </c>
       <c r="L29" s="12" t="inlineStr">
@@ -4050,7 +4056,7 @@
       <c r="J36" s="19" t="n"/>
       <c r="K36" s="12" t="inlineStr">
         <is>
-          <t>Derived from workout history + MQTT event timestamps.</t>
+          <t>Derived from workout history and cloud-synced workout event timestamps (transport per row 34 — currently an open gap).</t>
         </is>
       </c>
       <c r="L36" s="12" t="inlineStr">
@@ -4428,7 +4434,7 @@
       </c>
       <c r="K42" s="12" t="inlineStr">
         <is>
-          <t>Valinor Workout Player app; GlassOS Sindarin (brainboard bridge for speed/incline sensors); MQTT bio channel.</t>
+          <t>Valinor Workout Player app; GlassOS Sindarin (brainboard bridge for speed/incline sensors). Cloud transport for biometrics: see row 34 (open gap).</t>
         </is>
       </c>
       <c r="L42" s="12" t="inlineStr">
@@ -4438,7 +4444,7 @@
       </c>
       <c r="M42" s="12" t="inlineStr">
         <is>
-          <t>CONFIRMED (Workout Player component present in Club-2026-03 build; MQTT biometrics stream confirmed).</t>
+          <t>CONFIRMED (Workout Player component present in Club-2026-03 build). Prior 'MQTT biometrics stream confirmed' claim retracted 10/2/26 — MQTT is not implemented on current product.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scrub two more MQTT access-path cells (assets 4 and 33)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0158eT26M2Dsi3JDmdySDo5Y
</commit_message>
<xml_diff>
--- a/en18031_asset_inventory/merged_for_import_2026-10-02.xlsx
+++ b/en18031_asset_inventory/merged_for_import_2026-10-02.xlsx
@@ -856,9 +856,9 @@
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1" s="26">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>3. Residual MQTT mentions scrubbed from Asset Inventory rows 11, 19, 29, 36, 42 (assets 10, 18, 28, 35, 41). Current product does not use MQTT. Where a transport/endpoint cell is concerned, a one-line 'Future note' records that a proposed ToG project may add an MQTT-like service, explicitly out of current scope, so the claim is not re-introduced by mistake.</t>
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>3. Residual MQTT mentions scrubbed from Asset Inventory rows 5, 11, 19, 29, 34, 36, 42 (assets 4, 10, 18, 28, 33, 35, 41). Current product does not use MQTT. Where a transport/endpoint cell is concerned, a one-line 'Future note' records that a proposed ToG project may add an MQTT-like service, explicitly out of current scope, so the claim is not re-introduced by mistake.</t>
         </is>
       </c>
     </row>
@@ -2154,7 +2154,7 @@
       </c>
       <c r="L5" s="12" t="inlineStr">
         <is>
-          <t>Valinor cloud client (OkHttp GraphQL); MQTT client (mqtt-client-api).</t>
+          <t>Valinor cloud client (OkHttp GraphQL over HTTPS). (Prior 'MQTT client (mqtt-client-api)' reference retracted 10/2/26 — not in current product.)</t>
         </is>
       </c>
       <c r="M5" s="12" t="inlineStr">
@@ -3935,7 +3935,7 @@
       </c>
       <c r="L34" s="12" t="inlineStr">
         <is>
-          <t>BLE (HRM strap/grip sensors); MQTT; cloud sync.</t>
+          <t>BLE (HRM strap/grip sensors); cloud sync (transport mechanism is an open gap — see col M).</t>
         </is>
       </c>
       <c r="M34" s="21" t="inlineStr">

</xml_diff>

<commit_message>
Scrub MQTT from Interfaces and Where to Look tabs
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0158eT26M2Dsi3JDmdySDo5Y
</commit_message>
<xml_diff>
--- a/en18031_asset_inventory/merged_for_import_2026-10-02.xlsx
+++ b/en18031_asset_inventory/merged_for_import_2026-10-02.xlsx
@@ -582,7 +582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A45"/>
+  <dimension ref="A1:A46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="150" customWidth="1" style="26" min="1" max="1"/>
@@ -862,7 +862,13 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="15.75" customHeight="1" s="26"/>
+    <row r="46" ht="15.75" customHeight="1" s="26">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>4. Same MQTT scrub applied to Interfaces row 11 (Cloud backend connection) and Where to Look step 7 (Cloud link).</t>
+        </is>
+      </c>
+    </row>
     <row r="47" ht="15.75" customHeight="1" s="26"/>
     <row r="48" ht="15.75" customHeight="1" s="26"/>
     <row r="49" ht="15.75" customHeight="1" s="26"/>
@@ -8868,7 +8874,7 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Telemetry, account sync, OTA delivery, GraphQL API, MQTT event bus (including special-category biometric data).</t>
+          <t>Telemetry, account sync, OTA delivery, GraphQL API over HTTPS (carries special-category biometric data). Real-time transport, if any beyond GraphQL sync, is an open gap (Asset Inventory row 34).</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -8888,7 +8894,7 @@
       </c>
       <c r="H11" s="12" t="inlineStr">
         <is>
-          <t>Primary remote interface for nearly all Security, Network, and Privacy assets in this register — see Event Bus over MQTT and MQTT User Biometrics Confluence pages.</t>
+          <t>Primary remote interface for nearly all Security, Network, and Privacy assets in this register. Prior reference to the Event Bus over MQTT / MQTT User Biometrics Confluence pages retracted 10/2/26 — those describe a proposed future ToG project, not current Valinor. Future note: a proposed ToG tablet project may add an MQTT-like pub/sub service; NOT in current Xenon/Cesium scope and excluded from this assessment.</t>
         </is>
       </c>
     </row>
@@ -10155,12 +10161,12 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>TLS keys, API/MQTT/OAuth tokens, cloud endpoint config, personal data in transit</t>
+          <t>TLS keys, API/OAuth tokens, cloud endpoint config, personal data in transit</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>iFIT: GraphQL HTTPS API + MQTT-over-TLS (mqtt-client-api/mqtt-glassos-bridge). Certificate pinning status not confirmed — recommend explicit check.</t>
+          <t>iFIT: GraphQL HTTPS API (OkHttp). Certificate pinning status not confirmed — recommend explicit check. (Prior 'MQTT-over-TLS' reference retracted 10/2/26. Future note: a proposed ToG tablet project may add an MQTT-like pub/sub service; NOT in current Xenon/Cesium scope and excluded from this assessment.)</t>
         </is>
       </c>
     </row>

</xml_diff>